<commit_message>
Regenerate result tables with share-based indicators
All tables are rebuilt by 00_master.do from raw data. Tables 20, 21,
22 and 30 change only in their "generated by" header line. Paper 19
tables now hold AEI work shares for Korea and the world (no counts), and
paper 23, 25-29, 31 and 32 tables use shares, RU1-RU2 and indicator D
(new 27_dstats, 27_top_d, 19_b3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/table/26_kor_task_top30_conv.xlsx
+++ b/results/table/26_kor_task_top30_conv.xlsx
@@ -102,16 +102,16 @@
     <t>Apply mathematical theories and techniques to the solution of practical problems in business, engineering, the sciences, or other fields.</t>
   </si>
   <si>
-    <t>Archive documents, conduct research, and read copy, using the internet and various computer programs.</t>
-  </si>
-  <si>
     <t>Develop communications materials, advertisements, presentations, or public relations initiatives to promote awareness of products and services.</t>
   </si>
   <si>
     <t>Create graphs, charts, or other visualizations to convey the results of data analysis using specialized software.</t>
   </si>
   <si>
-    <t>Develop new visual design concepts and modify concepts based on stakeholder feedback.</t>
+    <t>Electronically sort and compile text and numerical data, retrieving, updating, and merging documents as required.</t>
+  </si>
+  <si>
+    <t>Compose business correspondence for supervisors, managers, and professionals.</t>
   </si>
   <si>
     <t>O*NET-SOC 코드</t>
@@ -195,16 +195,16 @@
     <t>15-2021.00</t>
   </si>
   <si>
-    <t>43-9081.00</t>
-  </si>
-  <si>
     <t>11-2011.00</t>
   </si>
   <si>
     <t>15-2051.00</t>
   </si>
   <si>
-    <t>15-1255.00</t>
+    <t>43-9022.00</t>
+  </si>
+  <si>
+    <t>43-9041.00</t>
   </si>
   <si>
     <t>직업(O*NET-SOC)</t>
@@ -288,16 +288,16 @@
     <t>Mathematicians</t>
   </si>
   <si>
-    <t>Proofreaders and Copy Markers</t>
-  </si>
-  <si>
     <t>Advertising and Promotions Managers</t>
   </si>
   <si>
     <t>Data Scientists</t>
   </si>
   <si>
-    <t>Web and Digital Interface Designers</t>
+    <t>Word Processors and Typists</t>
+  </si>
+  <si>
+    <t>Insurance Claims and Policy Processing Clerks</t>
   </si>
   <si>
     <t>SOC 2018 6자리</t>
@@ -381,16 +381,16 @@
     <t>15-2021</t>
   </si>
   <si>
-    <t>43-9081</t>
-  </si>
-  <si>
     <t>11-2011</t>
   </si>
   <si>
     <t>15-2051</t>
   </si>
   <si>
-    <t>15-1255</t>
+    <t>43-9022</t>
+  </si>
+  <si>
+    <t>43-9041</t>
   </si>
   <si>
     <t>SOC 대분류</t>
@@ -459,19 +459,19 @@
     <t>Computer and Mathematical</t>
   </si>
   <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Computer and Mathematical</t>
+  </si>
+  <si>
     <t>Office and Administrative Support</t>
   </si>
   <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>Computer and Mathematical</t>
-  </si>
-  <si>
-    <t>월평균 업무용 대화 수(K = 3)</t>
-  </si>
-  <si>
-    <t>한국 task 대화량 중 비중(%)</t>
+    <t>한국 업무용 대화 중 비중(%, 두 달 단순평균)</t>
+  </si>
+  <si>
+    <t>공개 task 대화 비중 합 중 비중(%)</t>
   </si>
   <si>
     <t>누적 비중(%)</t>
@@ -486,7 +486,7 @@
     <t>대화당 절감 시간(분, GLOBAL)</t>
   </si>
   <si>
-    <t>월평균 절감 시간(시간, K = 3)</t>
+    <t>비중 × 대화당 절감 시간(분, 두 달 평균)</t>
   </si>
 </sst>
 </file>
@@ -602,13 +602,13 @@
         <v>127</v>
       </c>
       <c r="H2" s="1">
-        <v>24785912.977437481</v>
+        <v>7.1607767845261572</v>
       </c>
       <c r="I2" s="1">
-        <v>6.8416174972868493</v>
+        <v>7.1635009398374274</v>
       </c>
       <c r="J2" s="1">
-        <v>6.8416174972868493</v>
+        <v>7.1635009398374274</v>
       </c>
       <c r="K2" s="1">
         <v>5.1550000000000002</v>
@@ -620,7 +620,7 @@
         <v>105.64036307053942</v>
       </c>
       <c r="N2" s="1">
-        <v>43639880.766188174</v>
+        <v>7.5646705938443315</v>
       </c>
     </row>
     <row r="3">
@@ -646,13 +646,13 @@
         <v>128</v>
       </c>
       <c r="H3" s="1">
-        <v>9535718.8834685683</v>
+        <v>2.7548622458269194</v>
       </c>
       <c r="I3" s="1">
-        <v>2.6321298401125937</v>
+        <v>2.7559102707611705</v>
       </c>
       <c r="J3" s="1">
-        <v>9.473747337399443</v>
+        <v>9.9194112105985983</v>
       </c>
       <c r="K3" s="1">
         <v>3.7749999999999999</v>
@@ -664,7 +664,7 @@
         <v>107.09279229711142</v>
       </c>
       <c r="N3" s="1">
-        <v>17020112.696515709</v>
+        <v>2.9502589029949617</v>
       </c>
     </row>
     <row r="4">
@@ -690,13 +690,13 @@
         <v>129</v>
       </c>
       <c r="H4" s="1">
-        <v>9082065.4832133111</v>
+        <v>2.6239789349591494</v>
       </c>
       <c r="I4" s="1">
-        <v>2.5069085886817768</v>
+        <v>2.624977168302741</v>
       </c>
       <c r="J4" s="1">
-        <v>11.980655926081219</v>
+        <v>12.544388378901338</v>
       </c>
       <c r="K4" s="1">
         <v>1.8849999999999998</v>
@@ -708,7 +708,7 @@
         <v>46.02524752475248</v>
       </c>
       <c r="N4" s="1">
-        <v>6966738.5316817239</v>
+        <v>1.2076927998123124</v>
       </c>
     </row>
     <row r="5">
@@ -734,13 +734,13 @@
         <v>130</v>
       </c>
       <c r="H5" s="1">
-        <v>6141277.0863395296</v>
+        <v>1.7742393107834167</v>
       </c>
       <c r="I5" s="1">
-        <v>1.695167283441791</v>
+        <v>1.7749142799365372</v>
       </c>
       <c r="J5" s="1">
-        <v>13.67582320952301</v>
+        <v>14.319302658837875</v>
       </c>
       <c r="K5" s="1">
         <v>1.28</v>
@@ -752,7 +752,7 @@
         <v>189.72057971014488</v>
       </c>
       <c r="N5" s="1">
-        <v>19418777.483016081</v>
+        <v>3.3660971058635774</v>
       </c>
     </row>
     <row r="6">
@@ -778,13 +778,13 @@
         <v>131</v>
       </c>
       <c r="H6" s="1">
-        <v>6137561.2074999493</v>
+        <v>1.7732203161545261</v>
       </c>
       <c r="I6" s="1">
-        <v>1.6941415951118994</v>
+        <v>1.7738948976542237</v>
       </c>
       <c r="J6" s="1">
-        <v>15.369964804634909</v>
+        <v>16.0931975564921</v>
       </c>
       <c r="K6" s="1">
         <v>1.2749999999999999</v>
@@ -796,7 +796,7 @@
         <v>461.74046979865761</v>
       </c>
       <c r="N6" s="1">
-        <v>47232673.256150715</v>
+        <v>8.1876758183771514</v>
       </c>
     </row>
     <row r="7">
@@ -822,13 +822,13 @@
         <v>132</v>
       </c>
       <c r="H7" s="1">
-        <v>5399002.1919227308</v>
+        <v>1.5598167716812272</v>
       </c>
       <c r="I7" s="1">
-        <v>1.4902782841920343</v>
+        <v>1.5604101686367595</v>
       </c>
       <c r="J7" s="1">
-        <v>16.860243088826945</v>
+        <v>17.653607725128861</v>
       </c>
       <c r="K7" s="1">
         <v>1.125</v>
@@ -840,7 +840,7 @@
         <v>205.60397849462368</v>
       </c>
       <c r="N7" s="1">
-        <v>18500938.84267512</v>
+        <v>3.2070453398030039</v>
       </c>
     </row>
     <row r="8">
@@ -866,13 +866,13 @@
         <v>133</v>
       </c>
       <c r="H8" s="1">
-        <v>5065623.0890156049</v>
+        <v>1.4634465022651735</v>
       </c>
       <c r="I8" s="1">
-        <v>1.3982561623619676</v>
+        <v>1.4640032373348271</v>
       </c>
       <c r="J8" s="1">
-        <v>18.258499251188912</v>
+        <v>19.117610962463687</v>
       </c>
       <c r="K8" s="1">
         <v>2.0049999999999999</v>
@@ -884,7 +884,7 @@
         <v>260.53200743494426</v>
       </c>
       <c r="N8" s="1">
-        <v>21995949.204833984</v>
+        <v>3.8127465500879332</v>
       </c>
     </row>
     <row r="9">
@@ -910,13 +910,13 @@
         <v>134</v>
       </c>
       <c r="H9" s="1">
-        <v>4867141.0315156672</v>
+        <v>1.4060906459724036</v>
       </c>
       <c r="I9" s="1">
-        <v>1.3434694648243304</v>
+        <v>1.4066255613058394</v>
       </c>
       <c r="J9" s="1">
-        <v>19.601968716013243</v>
+        <v>20.524236523769527</v>
       </c>
       <c r="K9" s="1">
         <v>1.0149999999999999</v>
@@ -928,7 +928,7 @@
         <v>267.54191780821918</v>
       </c>
       <c r="N9" s="1">
-        <v>21702737.430246264</v>
+        <v>3.7618818803565466</v>
       </c>
     </row>
     <row r="10">
@@ -954,13 +954,13 @@
         <v>134</v>
       </c>
       <c r="H10" s="1">
-        <v>4607301.4081817716</v>
+        <v>1.3310903981732902</v>
       </c>
       <c r="I10" s="1">
-        <v>1.2717463326117764</v>
+        <v>1.3315967813614662</v>
       </c>
       <c r="J10" s="1">
-        <v>20.873715048625019</v>
+        <v>21.855833305130993</v>
       </c>
       <c r="K10" s="1">
         <v>0.95999999999999996</v>
@@ -972,7 +972,7 @@
         <v>202.47632653061225</v>
       </c>
       <c r="N10" s="1">
-        <v>15547824.40579937</v>
+        <v>2.6951429410229775</v>
       </c>
     </row>
     <row r="11">
@@ -998,13 +998,13 @@
         <v>134</v>
       </c>
       <c r="H11" s="1">
-        <v>4584917.358793376</v>
+        <v>1.3246507337856774</v>
       </c>
       <c r="I11" s="1">
-        <v>1.2655676978326102</v>
+        <v>1.3251546671494179</v>
       </c>
       <c r="J11" s="1">
-        <v>22.139282746457631</v>
+        <v>23.180987972280413</v>
       </c>
       <c r="K11" s="1">
         <v>0.95500000000000007</v>
@@ -1016,7 +1016,7 @@
         <v>158.07417582417582</v>
       </c>
       <c r="N11" s="1">
-        <v>12079283.878553668</v>
+        <v>2.0939307299806069</v>
       </c>
     </row>
     <row r="12">
@@ -1042,13 +1042,13 @@
         <v>135</v>
       </c>
       <c r="H12" s="1">
-        <v>4182731.6922703544</v>
+        <v>1.2084102779650587</v>
       </c>
       <c r="I12" s="1">
-        <v>1.1545530059087479</v>
+        <v>1.2088699902806312</v>
       </c>
       <c r="J12" s="1">
-        <v>23.29383575236638</v>
+        <v>24.389857962561045</v>
       </c>
       <c r="K12" s="1">
         <v>0.87</v>
@@ -1060,7 +1060,7 @@
         <v>304.86395721925129</v>
       </c>
       <c r="N12" s="1">
-        <v>21252735.594865263</v>
+        <v>3.6840073928484323</v>
       </c>
     </row>
     <row r="13">
@@ -1086,13 +1086,13 @@
         <v>135</v>
       </c>
       <c r="H13" s="1">
-        <v>3995774.866820801</v>
+        <v>1.1544329783791754</v>
       </c>
       <c r="I13" s="1">
-        <v>1.1029476004755403</v>
+        <v>1.1548721562538933</v>
       </c>
       <c r="J13" s="1">
-        <v>24.396783352841922</v>
+        <v>25.54473011881494</v>
       </c>
       <c r="K13" s="1">
         <v>0.83000000000000007</v>
@@ -1104,7 +1104,7 @@
         <v>306.67647668393784</v>
       </c>
       <c r="N13" s="1">
-        <v>20423502.62964724</v>
+        <v>3.5403743837707005</v>
       </c>
     </row>
     <row r="14">
@@ -1130,13 +1130,13 @@
         <v>136</v>
       </c>
       <c r="H14" s="1">
-        <v>3915188.5552156228</v>
+        <v>1.1311619557796095</v>
       </c>
       <c r="I14" s="1">
-        <v>1.0807034846335424</v>
+        <v>1.1315922807209489</v>
       </c>
       <c r="J14" s="1">
-        <v>25.477486837475464</v>
+        <v>26.676322399535888</v>
       </c>
       <c r="K14" s="1">
         <v>0.69999999999999996</v>
@@ -1148,7 +1148,7 @@
         <v>181.88134328358211</v>
       </c>
       <c r="N14" s="1">
-        <v>11868329.22718541</v>
+        <v>2.0573725598847932</v>
       </c>
     </row>
     <row r="15">
@@ -1174,13 +1174,13 @@
         <v>137</v>
       </c>
       <c r="H15" s="1">
-        <v>3887410.5631533712</v>
+        <v>1.1231075234587138</v>
       </c>
       <c r="I15" s="1">
-        <v>1.0730359681411867</v>
+        <v>1.1235347842737373</v>
       </c>
       <c r="J15" s="1">
-        <v>26.550522805616652</v>
+        <v>27.799857183809625</v>
       </c>
       <c r="K15" s="1">
         <v>0.81000000000000005</v>
@@ -1192,7 +1192,7 @@
         <v>283.07342857142862</v>
       </c>
       <c r="N15" s="1">
-        <v>18340377.272943549</v>
+        <v>3.179218973198243</v>
       </c>
     </row>
     <row r="16">
@@ -1218,13 +1218,13 @@
         <v>137</v>
       </c>
       <c r="H16" s="1">
-        <v>3576353.5925924797</v>
+        <v>1.0332555544728821</v>
       </c>
       <c r="I16" s="1">
-        <v>0.98717539022421963</v>
+        <v>1.0336486331417634</v>
       </c>
       <c r="J16" s="1">
-        <v>27.537698195840871</v>
+        <v>28.833505816951387</v>
       </c>
       <c r="K16" s="1">
         <v>0.745</v>
@@ -1236,7 +1236,7 @@
         <v>148.50717741935486</v>
       </c>
       <c r="N16" s="1">
-        <v>8851902.9581579752</v>
+        <v>1.5344586594763818</v>
       </c>
     </row>
     <row r="17">
@@ -1262,13 +1262,13 @@
         <v>137</v>
       </c>
       <c r="H17" s="1">
-        <v>3337106.5607441468</v>
+        <v>0.9641470842804114</v>
       </c>
       <c r="I17" s="1">
-        <v>0.92113639941692094</v>
+        <v>0.96451387219735407</v>
       </c>
       <c r="J17" s="1">
-        <v>28.458834595257791</v>
+        <v>29.798019689148742</v>
       </c>
       <c r="K17" s="1">
         <v>0.69500000000000006</v>
@@ -1280,7 +1280,7 @@
         <v>171.50999999999996</v>
       </c>
       <c r="N17" s="1">
-        <v>9539119.1038871408</v>
+        <v>1.6536086642493331</v>
       </c>
     </row>
     <row r="18">
@@ -1306,13 +1306,13 @@
         <v>138</v>
       </c>
       <c r="H18" s="1">
-        <v>3279909.7801837362</v>
+        <v>0.94760279487679888</v>
       </c>
       <c r="I18" s="1">
-        <v>0.90534845991165447</v>
+        <v>0.94796328889362358</v>
       </c>
       <c r="J18" s="1">
-        <v>29.364183055169445</v>
+        <v>30.745982978042367</v>
       </c>
       <c r="K18" s="1">
         <v>1.4849999999999999</v>
@@ -1324,7 +1324,7 @@
         <v>103.0949295774648</v>
       </c>
       <c r="N18" s="1">
-        <v>5635701.1301413383</v>
+        <v>0.97693043405232394</v>
       </c>
     </row>
     <row r="19">
@@ -1350,13 +1350,13 @@
         <v>139</v>
       </c>
       <c r="H19" s="1">
-        <v>2936221.3773047999</v>
+        <v>0.84831090253783448</v>
       </c>
       <c r="I19" s="1">
-        <v>0.81048067784159072</v>
+        <v>0.84863362320352409</v>
       </c>
       <c r="J19" s="1">
-        <v>30.174663733011034</v>
+        <v>31.594616601245892</v>
       </c>
       <c r="K19" s="1">
         <v>0.60999999999999999</v>
@@ -1368,7 +1368,7 @@
         <v>56.823846153846148</v>
       </c>
       <c r="N19" s="1">
-        <v>2780789.8636267036</v>
+        <v>0.48204288216440283</v>
       </c>
     </row>
     <row r="20">
@@ -1394,13 +1394,13 @@
         <v>140</v>
       </c>
       <c r="H20" s="1">
-        <v>2854671.2896612436</v>
+        <v>0.82472479297733547</v>
       </c>
       <c r="I20" s="1">
-        <v>0.78797053237971826</v>
+        <v>0.82503854084194983</v>
       </c>
       <c r="J20" s="1">
-        <v>30.962634265390751</v>
+        <v>32.419655142087841</v>
       </c>
       <c r="K20" s="1">
         <v>0.59499999999999997</v>
@@ -1412,7 +1412,7 @@
         <v>52.138405797101456</v>
       </c>
       <c r="N20" s="1">
-        <v>2480633.5019615479</v>
+        <v>0.429998359271828</v>
       </c>
     </row>
     <row r="21">
@@ -1438,13 +1438,13 @@
         <v>141</v>
       </c>
       <c r="H21" s="1">
-        <v>2769182.9473662069</v>
+        <v>0.80006088362235761</v>
       </c>
       <c r="I21" s="1">
-        <v>0.76437331653408125</v>
+        <v>0.80036524866138103</v>
       </c>
       <c r="J21" s="1">
-        <v>31.727007581924831</v>
+        <v>33.22002039074922</v>
       </c>
       <c r="K21" s="1">
         <v>0.57499999999999996</v>
@@ -1456,7 +1456,7 @@
         <v>192.06481203007516</v>
       </c>
       <c r="N21" s="1">
-        <v>8864376.7043796666</v>
+        <v>1.5366354322554394</v>
       </c>
     </row>
     <row r="22">
@@ -1482,13 +1482,13 @@
         <v>142</v>
       </c>
       <c r="H22" s="1">
-        <v>2767671.0455522919</v>
+        <v>0.79961810219164109</v>
       </c>
       <c r="I22" s="1">
-        <v>0.76395598859810088</v>
+        <v>0.79992229878449972</v>
       </c>
       <c r="J22" s="1">
-        <v>32.490963570522929</v>
+        <v>34.019942689533721</v>
       </c>
       <c r="K22" s="1">
         <v>0.38500000000000001</v>
@@ -1500,7 +1500,7 @@
         <v>308.98391304347837</v>
       </c>
       <c r="N22" s="1">
-        <v>14252763.827864703</v>
+        <v>2.4706913015557324</v>
       </c>
     </row>
     <row r="23">
@@ -1526,13 +1526,13 @@
         <v>143</v>
       </c>
       <c r="H23" s="1">
-        <v>2709976.5374944303</v>
+        <v>0.78290906332203203</v>
       </c>
       <c r="I23" s="1">
-        <v>0.74803066213603597</v>
+        <v>0.78320690333957022</v>
       </c>
       <c r="J23" s="1">
-        <v>33.238994232658968</v>
+        <v>34.803149592873289</v>
       </c>
       <c r="K23" s="1">
         <v>0.56499999999999995</v>
@@ -1544,7 +1544,7 @@
         <v>232.74493670886076</v>
       </c>
       <c r="N23" s="1">
-        <v>10512221.96169398</v>
+        <v>1.8221812039167982</v>
       </c>
     </row>
     <row r="24">
@@ -1570,13 +1570,13 @@
         <v>144</v>
       </c>
       <c r="H24" s="1">
-        <v>2666682.383957386</v>
+        <v>0.77049740441456727</v>
       </c>
       <c r="I24" s="1">
-        <v>0.73608024341880351</v>
+        <v>0.77079052269764115</v>
       </c>
       <c r="J24" s="1">
-        <v>33.975074476077772</v>
+        <v>35.573940115570927</v>
       </c>
       <c r="K24" s="1">
         <v>1.0600000000000001</v>
@@ -1588,7 +1588,7 @@
         <v>212.67073059360729</v>
       </c>
       <c r="N24" s="1">
-        <v>9452088.180955328</v>
+        <v>1.638622459173241</v>
       </c>
     </row>
     <row r="25">
@@ -1614,13 +1614,13 @@
         <v>145</v>
       </c>
       <c r="H25" s="1">
-        <v>2638883.1819430068</v>
+        <v>0.76238471924105944</v>
       </c>
       <c r="I25" s="1">
-        <v>0.72840687237593249</v>
+        <v>0.76267475123683959</v>
       </c>
       <c r="J25" s="1">
-        <v>34.703481348453707</v>
+        <v>36.336614866807764</v>
       </c>
       <c r="K25" s="1">
         <v>0.55000000000000004</v>
@@ -1632,7 +1632,7 @@
         <v>432.61897727272725</v>
       </c>
       <c r="N25" s="1">
-        <v>19027182.388573062</v>
+        <v>3.2982209752642246</v>
       </c>
     </row>
     <row r="26">
@@ -1658,13 +1658,13 @@
         <v>146</v>
       </c>
       <c r="H26" s="1">
-        <v>2543776.767021744</v>
+        <v>0.73496052179805038</v>
       </c>
       <c r="I26" s="1">
-        <v>0.70215479471303388</v>
+        <v>0.73524012087916635</v>
       </c>
       <c r="J26" s="1">
-        <v>35.405636143166738</v>
+        <v>37.071854987686933</v>
       </c>
       <c r="K26" s="1">
         <v>1.01</v>
@@ -1676,7 +1676,7 @@
         <v>452.46565217391304</v>
       </c>
       <c r="N26" s="1">
-        <v>19182860.231255691</v>
+        <v>3.3254439181743427</v>
       </c>
     </row>
     <row r="27">
@@ -1702,13 +1702,13 @@
         <v>147</v>
       </c>
       <c r="H27" s="1">
-        <v>2535947.0765769617</v>
+        <v>0.73272524337704659</v>
       </c>
       <c r="I27" s="1">
-        <v>0.69999357728303147</v>
+        <v>0.73300399209712408</v>
       </c>
       <c r="J27" s="1">
-        <v>36.10562972044977</v>
+        <v>37.804858979784058</v>
       </c>
       <c r="K27" s="1">
         <v>0.52500000000000002</v>
@@ -1720,7 +1720,7 @@
         <v>80.164000000000001</v>
       </c>
       <c r="N27" s="1">
-        <v>3388194.3574452596</v>
+        <v>0.58738186410077564</v>
       </c>
     </row>
     <row r="28">
@@ -1728,7 +1728,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="1">
-        <v>20908</v>
+        <v>21222</v>
       </c>
       <c r="C28" t="s">
         <v>29</v>
@@ -1746,25 +1746,25 @@
         <v>148</v>
       </c>
       <c r="H28" s="1">
-        <v>2402000.6342112534</v>
+        <v>0.67986892494878481</v>
       </c>
       <c r="I28" s="1">
-        <v>0.66302054648837161</v>
+        <v>0.68012756567989496</v>
       </c>
       <c r="J28" s="1">
-        <v>36.768650266938138</v>
+        <v>38.484986545463954</v>
       </c>
       <c r="K28" s="1">
-        <v>0.41999999999999998</v>
+        <v>0.35999999999999999</v>
       </c>
       <c r="L28" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M28" s="1">
-        <v>378.90472727272726</v>
+        <v>354.1149999999999</v>
       </c>
       <c r="N28" s="1">
-        <v>15168823.253578881</v>
+        <v>2.4075178435823887</v>
       </c>
     </row>
     <row r="29">
@@ -1772,7 +1772,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="1">
-        <v>21222</v>
+        <v>21828</v>
       </c>
       <c r="C29" t="s">
         <v>30</v>
@@ -1790,25 +1790,25 @@
         <v>149</v>
       </c>
       <c r="H29" s="1">
-        <v>2353268.5946156881</v>
+        <v>0.66022220212407046</v>
       </c>
       <c r="I29" s="1">
-        <v>0.64956911643296089</v>
+        <v>0.66047336870454831</v>
       </c>
       <c r="J29" s="1">
-        <v>37.418219383371103</v>
+        <v>39.145459914168505</v>
       </c>
       <c r="K29" s="1">
-        <v>0.35999999999999999</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="L29" s="1">
         <v>2</v>
       </c>
       <c r="M29" s="1">
-        <v>354.1149999999999</v>
+        <v>426.73720000000003</v>
       </c>
       <c r="N29" s="1">
-        <v>13888795.139705569</v>
+        <v>2.8174137391225997</v>
       </c>
     </row>
     <row r="30">
@@ -1816,7 +1816,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="1">
-        <v>21828</v>
+        <v>799</v>
       </c>
       <c r="C30" t="s">
         <v>31</v>
@@ -1834,25 +1834,25 @@
         <v>150</v>
       </c>
       <c r="H30" s="1">
-        <v>2285225.0869251988</v>
+        <v>0.65397958184239846</v>
       </c>
       <c r="I30" s="1">
-        <v>0.6307871714944876</v>
+        <v>0.65422837355940722</v>
       </c>
       <c r="J30" s="1">
-        <v>38.049006554865592</v>
+        <v>39.799688287727911</v>
       </c>
       <c r="K30" s="1">
-        <v>0.47499999999999998</v>
+        <v>0.40500000000000003</v>
       </c>
       <c r="L30" s="1">
         <v>2</v>
       </c>
       <c r="M30" s="1">
-        <v>426.73720000000003</v>
+        <v>243.68779411764706</v>
       </c>
       <c r="N30" s="1">
-        <v>16253175.916070266</v>
+        <v>1.5936684169715529</v>
       </c>
     </row>
     <row r="31">
@@ -1860,7 +1860,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="1">
-        <v>21694</v>
+        <v>23334</v>
       </c>
       <c r="C31" t="s">
         <v>32</v>
@@ -1878,25 +1878,25 @@
         <v>150</v>
       </c>
       <c r="H31" s="1">
-        <v>2265569.6344841435</v>
+        <v>0.65359243178336612</v>
       </c>
       <c r="I31" s="1">
-        <v>0.62536170714059325</v>
+        <v>0.6538410762179051</v>
       </c>
       <c r="J31" s="1">
-        <v>38.674368262006183</v>
+        <v>40.453529363945819</v>
       </c>
       <c r="K31" s="1">
-        <v>0.47999999999999998</v>
+        <v>0.40500000000000003</v>
       </c>
       <c r="L31" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" s="1">
-        <v>429.08315789473687</v>
+        <v>74.94714285714285</v>
       </c>
       <c r="N31" s="1">
-        <v>16201962.88658135</v>
+        <v>0.48984885355215335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>